<commit_message>
big update, many bug fixes, view changes, + belgium, + portugal, and + european competitions.
</commit_message>
<xml_diff>
--- a/scoutingcost.xlsx
+++ b/scoutingcost.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jens\Documents\fussball-agent-app\FootballAgent\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4446998-F73F-4C05-9B59-85B3F3ED58C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFFF9D86-0C93-4825-8501-3151EF4899DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8EA1AADD-08EB-4841-99AA-B0094448DD60}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{8EA1AADD-08EB-4841-99AA-B0094448DD60}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="126">
   <si>
     <t># teams</t>
   </si>
@@ -354,14 +355,79 @@
   </si>
   <si>
     <t>LG-Saconnex</t>
+  </si>
+  <si>
+    <t xml:space="preserve">plan Fahrradreise </t>
+  </si>
+  <si>
+    <t>Startort</t>
+  </si>
+  <si>
+    <t>Endort</t>
+  </si>
+  <si>
+    <t>Distanz</t>
+  </si>
+  <si>
+    <t>Höhenmeter</t>
+  </si>
+  <si>
+    <t>Preis</t>
+  </si>
+  <si>
+    <t>Zürich</t>
+  </si>
+  <si>
+    <t>Dresden</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Usti Nad Labem</t>
+  </si>
+  <si>
+    <t>94.4 km</t>
+  </si>
+  <si>
+    <t>Zatec</t>
+  </si>
+  <si>
+    <t>104 km</t>
+  </si>
+  <si>
+    <t>Karlsbad</t>
+  </si>
+  <si>
+    <t>95.8 km</t>
+  </si>
+  <si>
+    <t>91.9 km</t>
+  </si>
+  <si>
+    <t>Pilsen</t>
+  </si>
+  <si>
+    <t>Furth im Wald</t>
+  </si>
+  <si>
+    <t>88.9 km</t>
+  </si>
+  <si>
+    <t>München</t>
+  </si>
+  <si>
+    <t>Winterthur</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="196" formatCode="0.0"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="&quot;CHF&quot;\ #,##0.00"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -403,14 +469,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="196" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -837,14 +905,14 @@
       <c r="A4" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="3">
         <v>33.222000000000001</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="3">
         <f>(23+27+41+80+60+26+25+29+23)/9</f>
         <v>37.111111111111114</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="3">
         <f>(75+65+35+33+25+30+23+63+40+20+20+35+18+28)/14</f>
         <v>36.428571428571431</v>
       </c>
@@ -852,7 +920,7 @@
         <f>(55+30+23+20+23+21+39)/9</f>
         <v>23.444444444444443</v>
       </c>
-      <c r="F4" s="2">
+      <c r="F4" s="3">
         <f>(70+54+25+58+42+48+26+20+20)/9</f>
         <v>40.333333333333336</v>
       </c>
@@ -864,11 +932,11 @@
         <f>(79+66+40+36+30+45+33+18+22)/9</f>
         <v>41</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="3">
         <f>(72+45+21+52+49+23+22+62+24)/9</f>
         <v>41.111111111111114</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="3">
         <f>(30+75+47+27+24+32+34+21+68+21+20+22)/12</f>
         <v>35.083333333333336</v>
       </c>
@@ -906,39 +974,39 @@
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B7" s="3">
+      <c r="B7" s="4">
         <f>((B4-30)*160)*((100-(50-B5))/100)*((100+B3)/100)</f>
         <v>663.06182400000023</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="4">
         <f t="shared" ref="C7:J7" si="0">((C4-30)*160)*((100-(50-C5))/100)*((100+C3)/100)</f>
         <v>1612.2311111111119</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="4">
         <f t="shared" si="0"/>
         <v>1465.7142857142862</v>
       </c>
-      <c r="E7" s="3">
+      <c r="E7" s="4">
         <f t="shared" si="0"/>
         <v>-1143.2888888888892</v>
       </c>
-      <c r="F7" s="3">
+      <c r="F7" s="4">
         <f t="shared" si="0"/>
         <v>2162.5600000000009</v>
       </c>
-      <c r="G7" s="3">
+      <c r="G7" s="4">
         <f t="shared" si="0"/>
         <v>2345.328</v>
       </c>
-      <c r="H7" s="3">
+      <c r="H7" s="4">
         <f t="shared" si="0"/>
         <v>2474.7360000000003</v>
       </c>
-      <c r="I7" s="3">
+      <c r="I7" s="4">
         <f t="shared" si="0"/>
         <v>2364.0888888888899</v>
       </c>
-      <c r="J7" s="3">
+      <c r="J7" s="4">
         <f t="shared" si="0"/>
         <v>1138.6666666666674</v>
       </c>
@@ -987,7 +1055,7 @@
       <c r="C10" t="s">
         <v>23</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="4" t="s">
         <v>30</v>
       </c>
       <c r="E10" t="s">
@@ -999,10 +1067,10 @@
       <c r="G10" t="s">
         <v>69</v>
       </c>
-      <c r="H10" s="3" t="s">
+      <c r="H10" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="I10" s="3" t="s">
+      <c r="I10" s="4" t="s">
         <v>82</v>
       </c>
       <c r="J10" t="s">
@@ -1141,7 +1209,7 @@
       <c r="F15" t="s">
         <v>55</v>
       </c>
-      <c r="G15" s="3" t="s">
+      <c r="G15" s="4" t="s">
         <v>45</v>
       </c>
       <c r="H15" t="s">
@@ -1153,7 +1221,7 @@
       <c r="J15" t="s">
         <v>97</v>
       </c>
-      <c r="L15" s="4"/>
+      <c r="L15" s="5"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
@@ -1250,10 +1318,288 @@
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A26" s="4"/>
+      <c r="A26" s="5"/>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B28">
+        <f>(B4-33.222)/(41.125-33.222)</f>
+        <v>0</v>
+      </c>
+      <c r="C28">
+        <f t="shared" ref="C28:J28" si="1">(C4-33.222)/(41.125-33.222)</f>
+        <v>0.49210567013932854</v>
+      </c>
+      <c r="D28">
+        <f t="shared" si="1"/>
+        <v>0.4057410386652448</v>
+      </c>
+      <c r="E28">
+        <f t="shared" si="1"/>
+        <v>-1.2371954391440667</v>
+      </c>
+      <c r="F28">
+        <f t="shared" si="1"/>
+        <v>0.89982706988907191</v>
+      </c>
+      <c r="G28">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="H28">
+        <f t="shared" si="1"/>
+        <v>0.98418322156143234</v>
+      </c>
+      <c r="I28">
+        <f t="shared" si="1"/>
+        <v>0.99824258017349288</v>
+      </c>
+      <c r="J28">
+        <f t="shared" si="1"/>
+        <v>0.23552237546923127</v>
+      </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="H30" s="4"/>
+      <c r="B30">
+        <f t="shared" ref="B30:D30" si="2">B28*3400 + 600</f>
+        <v>600</v>
+      </c>
+      <c r="C30">
+        <f t="shared" si="2"/>
+        <v>2273.1592784737168</v>
+      </c>
+      <c r="D30">
+        <f t="shared" si="2"/>
+        <v>1979.5195314618322</v>
+      </c>
+      <c r="E30">
+        <f>E28*3400 + 600</f>
+        <v>-3606.4644930898266</v>
+      </c>
+      <c r="F30">
+        <f t="shared" ref="F30:J30" si="3">F28*3400 + 600</f>
+        <v>3659.4120376228443</v>
+      </c>
+      <c r="G30">
+        <f t="shared" si="3"/>
+        <v>4000</v>
+      </c>
+      <c r="H30">
+        <f t="shared" si="3"/>
+        <v>3946.2229533088698</v>
+      </c>
+      <c r="I30">
+        <f t="shared" si="3"/>
+        <v>3994.0247725898757</v>
+      </c>
+      <c r="J30">
+        <f t="shared" si="3"/>
+        <v>1400.7760765953863</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94298849-AB24-4101-9D64-E52B1CE3075C}">
+  <dimension ref="A1:F15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="17.7109375" customWidth="1"/>
+    <col min="3" max="3" width="16.85546875" customWidth="1"/>
+    <col min="5" max="5" width="13" customWidth="1"/>
+    <col min="6" max="6" width="10.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D2" t="s">
+        <v>108</v>
+      </c>
+      <c r="E2" t="s">
+        <v>109</v>
+      </c>
+      <c r="F2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>21.7</v>
+      </c>
+      <c r="B3" t="s">
+        <v>111</v>
+      </c>
+      <c r="C3" t="s">
+        <v>112</v>
+      </c>
+      <c r="D3" t="s">
+        <v>113</v>
+      </c>
+      <c r="E3" t="s">
+        <v>113</v>
+      </c>
+      <c r="F3" s="6">
+        <f xml:space="preserve"> 63.06 * 0.922</f>
+        <v>58.141320000000007</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>22.7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C4" t="s">
+        <v>114</v>
+      </c>
+      <c r="D4" t="s">
+        <v>115</v>
+      </c>
+      <c r="E4">
+        <v>826</v>
+      </c>
+      <c r="F4" s="6">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>23.7</v>
+      </c>
+      <c r="B5" t="s">
+        <v>114</v>
+      </c>
+      <c r="C5" t="s">
+        <v>116</v>
+      </c>
+      <c r="D5" t="s">
+        <v>117</v>
+      </c>
+      <c r="E5">
+        <v>604</v>
+      </c>
+      <c r="F5" s="6">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>24.7</v>
+      </c>
+      <c r="B6" t="s">
+        <v>116</v>
+      </c>
+      <c r="C6" t="s">
+        <v>118</v>
+      </c>
+      <c r="D6" t="s">
+        <v>119</v>
+      </c>
+      <c r="E6">
+        <v>1119</v>
+      </c>
+      <c r="F6" s="6">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>25.7</v>
+      </c>
+      <c r="B7" t="s">
+        <v>118</v>
+      </c>
+      <c r="C7" t="s">
+        <v>121</v>
+      </c>
+      <c r="D7" t="s">
+        <v>120</v>
+      </c>
+      <c r="E7">
+        <v>1457</v>
+      </c>
+      <c r="F7" s="6">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>26.7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>121</v>
+      </c>
+      <c r="C8" t="s">
+        <v>122</v>
+      </c>
+      <c r="D8" t="s">
+        <v>123</v>
+      </c>
+      <c r="E8">
+        <v>1014</v>
+      </c>
+      <c r="F8" s="6"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>26.7</v>
+      </c>
+      <c r="B9" t="s">
+        <v>122</v>
+      </c>
+      <c r="C9" t="s">
+        <v>124</v>
+      </c>
+      <c r="F9" s="6">
+        <f xml:space="preserve"> 32 * 0.922</f>
+        <v>29.504000000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>27.7</v>
+      </c>
+      <c r="B10" t="s">
+        <v>124</v>
+      </c>
+      <c r="C10" t="s">
+        <v>125</v>
+      </c>
+      <c r="F10" s="6">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F11" s="6"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F12" s="6">
+        <f>SUM(F3:F10)</f>
+        <v>300.64531999999997</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F13" s="6"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F14" s="6"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F15" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>